<commit_message>
Add business scan report Excel: נהר פרת, ירושלים — 6 businesses found (indices 17031-17042)
</commit_message>
<xml_diff>
--- a/excel outputs/דוח נכסים לתאריך:27-08-2026.xlsx
+++ b/excel outputs/דוח נכסים לתאריך:27-08-2026.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="נכסים" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="עסקים" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,27 +26,71 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
     </font>
     <font>
-      <name val="Arial"/>
+      <color rgb="007B6000"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
       <color rgb="000563C1"/>
       <u val="single"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -54,20 +98,58 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="001F4E79"/>
+      </left>
+      <right style="thin">
+        <color rgb="001F4E79"/>
+      </right>
+      <top style="thin">
+        <color rgb="001F4E79"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="001F4E79"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -434,173 +516,393 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="23" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="17" customWidth="1" min="5" max="5"/>
-    <col width="36" customWidth="1" min="6" max="6"/>
-    <col width="50" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="7" max="7"/>
+    <col width="42" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>דוח עסקים לפי כתובת — 27-08-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>סריקה: רחוב נהר פרת, נחלאות, ירושלים | אינדקסים 17031–17042 | 6 עסקים מאומתים מתוך 12 כתובות שנסרקו</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>⚠️ בניינים אלו הם בניינים מגורים — ייתכן עסקים נוספים שאינם ברשומות ציבוריות | מספרי מקשר של זאפ לא נכללו</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
           <t>שם העסק</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>כתובת</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>שכונה</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>סוג עסק</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>דירוג אינדיקציה</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>קישור 1</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>קישור 2</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>קישור 3</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>חבד (בית הכנסת חבד מזרח)</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>יוסף נדבה 1, ירושלים</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>פסגת זאב מזרח</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>בית כנסת</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>https://easy.co.il/page/25964052</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>https://mypisga.co.il/bateycneset/%D7%97%D7%91%D7%93-%D7%9E%D7%96%D7%A8%D7%97</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>הילי חברה לבניה</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>יוסף נדבה 23, ירושלים</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>פסגת זאב מזרח</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>שיפוצים ובניה</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/80071101/48570</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>הפרח בגני</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>יוסף נדבה 53, ירושלים</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>פסגת זאב מזרח</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>פרחים וגינון</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>גבוה</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>https://www.d.co.il/35497550/11000</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr"/>
-      <c r="H4" s="2" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>כתובת (לפי הקישור)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>תחום / קטגוריה</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>טלפון (לפי הקישור)</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>כתובת אתר רשמי</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>קישור מקור 1</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>קישור מקור 2</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>קישור מקור 3</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>תאריך עדכניות</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="28" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>מקרוArt ציורי פנים וגוף</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>נהר פרת 17, ירושלים</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>ציורי פנים וגוף</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>דפי זהב</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I5" s="5" t="inlineStr">
+        <is>
+          <t>— (אין תאריך גלוי)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="28" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>אוגדן פיתוח ובניין</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>נהר פרת 19, ירושלים</t>
+        </is>
+      </c>
+      <c r="C6" s="7" t="inlineStr">
+        <is>
+          <t>שיפוצים ובנייה</t>
+        </is>
+      </c>
+      <c r="D6" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E6" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>תפוצות</t>
+        </is>
+      </c>
+      <c r="G6" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I6" s="7" t="inlineStr">
+        <is>
+          <t>— (אין תאריך גלוי)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="28" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>מ.ד. חפירות והשקעות בע"מ</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>נהר פרת 19, ירושלים</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>חפירות והשקעות</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>CheckID</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I7" s="5" t="inlineStr">
+        <is>
+          <t>— (אין תאריך גלוי)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="28" customHeight="1">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>חיים נדל"ן עסקי (מלכה חיים)</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>נהר פרת 20, ירושלים</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>תיווך נדל"ן</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E8" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>B144</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>דפי זהב</t>
+        </is>
+      </c>
+      <c r="H8" s="7" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I8" s="7" t="inlineStr">
+        <is>
+          <t>— (אין תאריך גלוי)</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="28" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>שיראל ותהילה קפוארה לנשים</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>נהר פרת 22, ירושלים</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>קפואירה</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>דפי זהב</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I9" s="5" t="inlineStr">
+        <is>
+          <t>— (אין תאריך גלוי)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="28" customHeight="1">
+      <c r="A10" s="9" t="inlineStr">
+        <is>
+          <t>ליברמן ישי (עו"ד)</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="inlineStr">
+        <is>
+          <t>נהר פרת 3, ירושלים</t>
+        </is>
+      </c>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>עורך דין ✅</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="F10" s="10" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="G10" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I10" s="9" t="inlineStr">
+        <is>
+          <t>— (אין תאריך גלוי)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>סה"כ עסקים שנמצאו: 6 | מקורות: B144, דפי זהב, Easy.co.il, CheckID, תפוצות | Easy.co.il לא אפשר חילוץ ישיר (חסום)</t>
+        </is>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A2:I2"/>
+    <mergeCell ref="A11:I11"/>
+  </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F4" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F5" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F6" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F7" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F8" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G8" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F9" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="G9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F10" r:id="rId8"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>